<commit_message>
Formulation v1.1: replace 18-MEA complex and Germaben II
- Cutissential Behenyl 18-MEA replaced by Incroquat Behenyl TMS-50
  (BTMS + cetyl alcohol + butylene glycol) 0.8% plus cetyl alcohol
  raised to 0.4%, keeping total cationics at 1.0% active and fatty
  alcohol at ~0.7%.
- Germaben II and separate phenoxyethanol replaced by Euxyl PE 9010
  (phenoxyethanol + ethylhexylglycerin) 1.0% plus potassium sorbate
  0.3%; pH target lowered to 4.8 so the sorbate works.
- Updated notes, process, QC, tuning, EU compliance table and label
  INCI in the xlsx, md and pdf; all three built from one data file.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UmFF3CgoK15mLAmmhMv9dF
</commit_message>
<xml_diff>
--- a/estel-18-plus/estel-18-plus-spray-formula.xlsx
+++ b/estel-18-plus/estel-18-plus-spray-formula.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="275">
-  <si>
-    <t xml:space="preserve">Рецептура: несмываемый спрей-молочко для волос типа ESTEL 18 PLUS (вариант для рынка ЕС, без D5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Однородная белая эмульсия на катионных ПАВ, вязкость около 100 мПа·с, pH 5,0. Дозировки: оценка по INCI оригинала и измерениям эталона (pH 5, плотность 1,01, вязкость около 100 мПа·с), требуют лабораторной проверки. Синим выделены вводимые значения (дозировки, активность сырья), чёрным: формулы.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="288">
+  <si>
+    <t xml:space="preserve">Рецептура: несмываемый спрей-молочко для волос типа ESTEL 18 PLUS (рынок ЕС, без D5). Версия 1.1 от 08.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Однородная белая эмульсия на катионных ПАВ, вязкость около 100 мПа·с, pH 4,8. Версия 1.1: комплекс 18-MEA заменён на Incroquat Behenyl TMS-50, Germaben II и феноксиэтанол заменены на Euxyl PE 9010 + сорбат калия. Дозировки: оценка по INCI оригинала и измерениям эталона (pH 5, плотность 1,01, вязкость около 100 мПа·с), требуют лабораторной проверки. Синим выделены вводимые значения (дозировки, активность сырья), чёрным: формулы.</t>
   </si>
   <si>
     <t xml:space="preserve">№</t>
@@ -87,7 +87,7 @@
     <t xml:space="preserve">Хелатор</t>
   </si>
   <si>
-    <t xml:space="preserve">Растворить первым</t>
+    <t xml:space="preserve">Растворить первым; также защищает сорбат от окисления</t>
   </si>
   <si>
     <t xml:space="preserve">Glycerin</t>
@@ -117,9 +117,6 @@
     <t xml:space="preserve">Увлажнитель, носитель</t>
   </si>
   <si>
-    <t xml:space="preserve">Ещё около 0,45 % приходит с Germaben II</t>
-  </si>
-  <si>
     <t xml:space="preserve">Betaine</t>
   </si>
   <si>
@@ -138,7 +135,7 @@
     <t xml:space="preserve">Актив: уход за кожей головы, укрепление</t>
   </si>
   <si>
-    <t xml:space="preserve">Стабилен при pH 5</t>
+    <t xml:space="preserve">Стабилен при pH 4,5–5</t>
   </si>
   <si>
     <t xml:space="preserve">Caffeine</t>
@@ -183,16 +180,16 @@
     <t xml:space="preserve">0,6 % активного. Растворитель грейда (изопропанол или этанол) указать в INCI. ЕС Annex III/287: не более 3 % в несмываемых средствах для волос</t>
   </si>
   <si>
-    <t xml:space="preserve">Behentrimonium Methosulfate (and) C10-40 Isoalkylamidopropylethyldimonium Ethosulfate (and) Cetyl Alcohol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cutissential Behenyl 18-MEA (Croda)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кондиционер, имитатор липида кутикулы 18-MEA, соэмульгатор и структурообразователь</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Состав по TDS: BTMS 20–30 %, C10-40 кват 10–20 %, остальное цетиловый спирт. Замена при отсутствии: Incroquat Behenyl TMS-50 (Croda) 1,0 %</t>
+    <t xml:space="preserve">Behentrimonium Methosulfate (and) Cetyl Alcohol (and) Butylene Glycol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incroquat Behenyl TMS-50 (Croda); аналоги: BTMS-50 других поставщиков с тем же INCI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Катионный эмульгатор и кондиционер, структурообразователь (замена комплекса 18-MEA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ориентировочно 50 % BTMS, ~37 % цетилового спирта, ~13 % бутиленгликоля (уточнить по TDS). Даёт 0,4 % BTMS и ~0,3 % цетилового спирта. Не заменять на BTMS-25 (Varisoft BT 85, Incroquat Behenyl TMS): там цетеариловый спирт, вязкость вырастет, INCI изменится</t>
   </si>
   <si>
     <t xml:space="preserve">Cetyl Alcohol</t>
@@ -204,7 +201,7 @@
     <t xml:space="preserve">Структурообразователь, регулятор вязкости</t>
   </si>
   <si>
-    <t xml:space="preserve">Диапазон 0,1–0,5 %: больше спирта, выше вязкость</t>
+    <t xml:space="preserve">0,4 % компенсирует меньшую долю жирного спирта в TMS-50 по сравнению с комплексом 18-MEA; итого жирного спирта ~0,7 %. Диапазон 0,2–0,6 %: больше спирта, выше вязкость</t>
   </si>
   <si>
     <t xml:space="preserve">C12-15 Alkyl Benzoate</t>
@@ -441,361 +438,391 @@
     <t xml:space="preserve">E</t>
   </si>
   <si>
+    <t xml:space="preserve">Phenoxyethanol (and) Ethylhexylglycerin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Euxyl PE 9010 (Schülke): феноксиэтанол 90 % + этилгексилглицерин 10 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Консервант широкого спектра с усилителем (замена феноксиэтанола 0,5 % и Germaben II 0,8 %)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Даёт феноксиэтанол 0,9 % (лимит ЕС 1,0 %, Annex V/29) и этилгексилглицерин 0,1 %. Аналог в одном компоненте: Optiphen Plus (Ashland) 1,0 % при pH ниже 6, тогда отдельный сорбат не нужен</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potassium Sorbate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сорбат калия, косметический; растворить в воде 1:5 перед вводом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Противогрибковый компонент (плесени, дрожжи)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Работает в виде недиссоциированной сорбиновой кислоты, поэтому pH 4,6–5,0. ЕС Annex V/4: не более 0,6 % в пересчёте на кислоту (здесь ~0,22 %). Вводить до корректировки pH; беречь массу от света, EDTA в рецептуре защищает от окисления</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PEG-40 Hydrogenated Castor Oil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kolliphor RH 40 / Eumulgin HRE 40 (BASF) / Croduret 40 (Croda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Солюбилизатор отдушки, стабильность распыления</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Смешать с отдушкой до прозрачности, затем ввести в массу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parfum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отдушка заказчика с IFRA-сертификатом и декларацией аллергенов</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отдушка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Аллергены в INCI по декларации поставщика. ЕС: порог 0,001 % для несмываемых; новый список аллергенов (Регл. 2023/1545) для новых продуктов с 31.07.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фаза F. Корректировка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lactic Acid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Молочная кислота 80 % (Purac HS 80, Corbion), вводить как 20 % водный раствор</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Регулятор pH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">q.s. до pH 4,8 ± 0,2; ориентир 0,15–0,35 % по кислоте 80 % (сорбат слегка подщелачивает)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ИТОГО</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сумма по фазам, % масс.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Масляная фаза без эмульгаторов (поз. 13–20)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Катионные ПАВ и цетиловый спирт, по сырью (поз. 10–12)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Источники по сырью: Croda (Incroquat Behenyl TMS-50), Momentive (Silsoft Q PMF), Dow (XIAMETER PMX-1503, OFX-0193, DOWSIL 556), Nouryon (ElfaMoist AC), Schülke (Euxyl PE 9010); составы по TDS поставщиков. Параметры эталона: измерения технолога-заказчика.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Порядок изготовления (лабораторный замес, роторно-статорный гомогенизатор)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Шаг</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стадия</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Операция</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фаза A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В воду при перемешивании ввести EDTA, затем глицерин, сорбитол, пропиленгликоль, бетаин, ниацинамид, кофеин; распылить гиалуронат. Нагреть до 75–80 °C, перемешивать до полного растворения.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фаза B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сплавить компоненты при 75–80 °C до однородного прозрачного расплава.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Эмульгирование</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ввести фазу B в фазу A при 75–80 °C под роторно-статорным гомогенизатором, 3–5 мин (лабораторно 3000–5000 об/мин). Перейти на якорную или лопастную мешалку, начать охлаждение.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фаза C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">При температуре не выше 40 °C ввести изододекан, гомогенизация 1–2 мин, закрытая ёмкость, без открытого огня.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фаза D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">При температуре не выше 40 °C ввести компоненты по одному, перемешивая до однородности после каждого.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фаза E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">При температуре не выше 35 °C ввести Euxyl PE 9010, затем раствор сорбата калия (1:5 в воде из рецептурного количества), затем отдушку, заранее смешанную с PEG-40 HCO.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фаза F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Довести pH до 4,8 ± 0,2 молочной кислотой (20 % раствор). Долить воду до 100 % с учётом потерь. Перемешивать 10 мин, удалить воздух (вакуум или отстаивание).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Контроль готового продукта (ориентиры под эталон)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Показатель</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Норма</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Внешний вид</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Белое однородное молочко без расслоения и комков</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pH (20 °C)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4,8 ± 0,2 (эталон 5,0; снижено, чтобы работал сорбат)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вязкость</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80–150 мПа·с (эталон: около 100; по методике технолога)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Плотность</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,00–1,01 г/см³ (эталон: 1,01; расчётная около 1,00)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Распыление</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Равномерный факел без крупных капель, помпа не забивается после 50 нажатий</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стабильность</t>
+  </si>
+  <si>
+    <t xml:space="preserve">По внутренним стандартам лаборатории; ориентир: центрифуга 3000 об/мин 30 мин, 3 цикла заморозки, 45 °C 1–3 мес</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Микробиология</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Challenge-тест по ISO 11930 обязателен для досье ЕС: новая система консервации без парабенов</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тонкая настройка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проблема</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Действие</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вязкость ниже целевой</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цетиловый спирт +0,1–0,2 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вязкость выше целевой</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цетиловый спирт −0,1 % или Behentrimonium Chloride −0,1 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отстой масла или сливки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Усилить гомогенизацию на стадии 3; Incroquat Behenyl TMS-50 до 1,2 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Помутнение, осадок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проверить совместимость анионных компонентов (гиалуронат, КМ-хитин, сорбат) с катионными; снизить их уровень</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не прошёл challenge-тест по плесени</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pH до 4,6; сорбат калия до 0,4 % (лимит 0,6 % как кислота) или перейти на Optiphen Plus 1,2 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Слишком тяжёлые волосы</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Снизить PMX-1503 до 1,0 % и Phenyl Trimethicone до 0,3 %; изододекан оставить</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отличия от оригинала и соответствие Регламенту (ЕС) 1223/2009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Что изменено относительно INCI оригинала</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Компонент</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Решение</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Основание</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cyclopentasiloxane (D5)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Исключён</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Регл. (ЕС) 2024/1328 (REACH, запись 70): D4, D5, D6 не более 0,1 % в несмываемых косметических средствах с 06.06.2027. Замена: XIAMETER PMX-1503 (диметиконол в линейном диметиконе) плюс изододекан как летучий носитель.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cutissential Behenyl 18-MEA (Behentrimonium Methosulfate + C10-40 Isoalkylamidopropylethyldimonium Ethosulfate + Cetyl Alcohol)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заменён</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Incroquat Behenyl TMS-50 (Behentrimonium Methosulfate, Cetyl Alcohol, Butylene Glycol) 0,8 % плюс цетиловый спирт 0,4 %. Та же функциональная пара «бегениловый кват + цетиловый спирт», но без специального 18-MEA-квата: суммарно катионных ПАВ 1,0 % активного и жирного спирта ~0,7 %, как в версии 1.0, поэтому вязкость и кондиционирование сохраняются. Уходит только заявление о восстановлении липида 18-MEA. В INCI: минус C10-40 кват, плюс Butylene Glycol.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Germaben II (Propylene Glycol, Diazolidinyl Urea, Methylparaben, Propylparaben) и Phenoxyethanol 0,5 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Заменены</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Euxyl PE 9010 (Phenoxyethanol 90 % + Ethylhexylglycerin 10 %) 1,0 % плюс Potassium Sorbate 0,3 %, pH 4,8. Причины: диазолидинилмочевина выделяет формальдегид (маркировка «выделяет формальдегид» по Регл. 2022/1181, контактный аллерген), парабены нежелательны для розницы ЕС, а феноксиэтанол уже был в составе. Новая система без парабенов, формальдегид-доноров и маркируемых аллергенов; сорбат закрывает плесени и дрожжи, слабое место феноксиэтанола. Общая нагрузка консервантов 1,3 %, как раньше.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CI 60730</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Эталон белый, по решению заказчика краситель не нужен.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Остальной состав</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сохранён</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Все остальные INCI оригинала сохранены; порядок INCI готового продукта изменится (см. раздел INCI).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Регуляторные лимиты ЕС и уровни в рецептуре</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вещество</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ссылка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Лимит / требование</t>
+  </si>
+  <si>
+    <t xml:space="preserve">В рецептуре</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annex III/287</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не более 3 % в несмываемых средствах для волос</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,60 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Behentrimonium Methosulfate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не нормируется</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ограничений в приложениях Регл. 1223/2009 нет</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,40 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annex VI/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не более 10 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,30 %</t>
+  </si>
+  <si>
     <t xml:space="preserve">Phenoxyethanol</t>
   </si>
   <si>
-    <t xml:space="preserve">Phenoxetol (Clariant) или аналог</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Консервант</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ЕС Annex V/29: не более 1,0 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propylene Glycol (and) Diazolidinyl Urea (and) Methylparaben (and) Propylparaben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Germaben II (Ashland)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Консервант, система оригинала</t>
-  </si>
-  <si>
-    <t xml:space="preserve">В продукте: Diazolidinyl Urea 0,24 % (лимит ЕС 0,5 %), Methylparaben 0,09 % (0,4 %), Propylparaben 0,02 % (0,14 %). ЕС Регл. 2022/1181: при свободном формальдегиде более 0,001 % нужна надпись «выделяет формальдегид»</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PEG-40 Hydrogenated Castor Oil</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kolliphor RH 40 / Eumulgin HRE 40 (BASF) / Croduret 40 (Croda)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Солюбилизатор отдушки, стабильность распыления</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Смешать с отдушкой до прозрачности, затем ввести в массу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Parfum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Отдушка заказчика с IFRA-сертификатом и декларацией аллергенов</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Отдушка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Аллергены в INCI по декларации поставщика. ЕС: порог 0,001 % для несмываемых; новый список аллергенов (Регл. 2023/1545) для новых продуктов с 31.07.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фаза F. Корректировка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Lactic Acid</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Молочная кислота 80 % (Purac HS 80, Corbion), вводить как 20 % водный раствор</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Регулятор pH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">q.s. до pH 5,0 ± 0,2; ориентир 0,10–0,25 % по кислоте 80 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ИТОГО</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сумма по фазам, % масс.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Масляная фаза без эмульгаторов (поз. 13–20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Катионные ПАВ и цетиловый спирт, по сырью (поз. 10–12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Источники по сырью: Croda (Cutissential Behenyl 18-MEA), Momentive (Silsoft Q PMF), Dow (XIAMETER PMX-1503, OFX-0193, DOWSIL 556), Nouryon (ElfaMoist AC), Ashland (Germaben II); составы по TDS поставщиков. Параметры эталона: измерения технолога-заказчика.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Порядок изготовления (лабораторный замес, роторно-статорный гомогенизатор)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Шаг</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стадия</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Операция</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фаза A</t>
-  </si>
-  <si>
-    <t xml:space="preserve">В воду при перемешивании ввести EDTA, затем глицерин, сорбитол, пропиленгликоль, бетаин, ниацинамид, кофеин; распылить гиалуронат. Нагреть до 75–80 °C, перемешивать до полного растворения.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фаза B</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сплавить компоненты при 75–80 °C до однородного прозрачного расплава.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Эмульгирование</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ввести фазу B в фазу A при 75–80 °C под роторно-статорным гомогенизатором, 3–5 мин (лабораторно 3000–5000 об/мин). Перейти на якорную или лопастную мешалку, начать охлаждение.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фаза C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">При температуре не выше 40 °C ввести изододекан, гомогенизация 1–2 мин, закрытая ёмкость, без открытого огня.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фаза D</t>
-  </si>
-  <si>
-    <t xml:space="preserve">При температуре не выше 40 °C ввести компоненты по одному, перемешивая до однородности после каждого.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фаза E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">При температуре не выше 35 °C ввести феноксиэтанол и Germaben II, затем отдушку, заранее смешанную с PEG-40 HCO.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фаза F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Довести pH до 5,0 ± 0,2 молочной кислотой (20 % раствор). Долить воду до 100 % с учётом потерь. Перемешивать 10 мин, удалить воздух (вакуум или отстаивание).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Контроль готового продукта (ориентиры под эталон)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Показатель</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Норма</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Внешний вид</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Белое однородное молочко без расслоения и комков</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pH (20 °C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">5,0 ± 0,3 (эталон: 5,0)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вязкость</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80–150 мПа·с (эталон: около 100; по методике технолога)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Плотность</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1,00–1,01 г/см³ (эталон: 1,01; расчётная около 1,00)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Распыление</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Равномерный факел без крупных капель, помпа не забивается после 50 нажатий</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стабильность</t>
-  </si>
-  <si>
-    <t xml:space="preserve">По внутренним стандартам лаборатории; ориентир: центрифуга 3000 об/мин 30 мин, 3 цикла заморозки, 45 °C 1–3 мес</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тонкая настройка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Проблема</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Действие</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вязкость ниже целевой</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цетиловый спирт +0,1–0,2 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вязкость выше целевой</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цетиловый спирт −0,1 % или Behentrimonium Chloride −0,1 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Отстой масла или сливки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Усилить гомогенизацию на стадии 3; Cutissential Behenyl 18-MEA до 1,5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Помутнение, осадок</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Проверить совместимость анионных компонентов (гиалуронат, КМ-хитин) с катионными; снизить их уровень</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Слишком тяжёлые волосы</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Снизить PMX-1503 до 1,0 % и Phenyl Trimethicone до 0,3 %; изододекан оставить</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Отличия от оригинала и соответствие Регламенту (ЕС) 1223/2009</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Что изменено относительно INCI оригинала</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Компонент</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Решение</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Основание</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cyclopentasiloxane (D5)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Исключён</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Регл. (ЕС) 2024/1328 (REACH, запись 70): D4, D5, D6 не более 0,1 % в несмываемых косметических средствах с 06.06.2027. Замена: XIAMETER PMX-1503 (диметиконол в линейном диметиконе) плюс изододекан как летучий носитель.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CI 60730</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Эталон белый, по решению заказчика краситель не нужен.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Остальной состав</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сохранён</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Все остальные INCI оригинала сохранены; порядок INCI готового продукта изменится (см. ниже).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Регуляторные лимиты ЕС и уровни в рецептуре</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вещество</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ссылка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Лимит / требование</t>
-  </si>
-  <si>
-    <t xml:space="preserve">В рецептуре</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex III/287</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 3 % в несмываемых средствах для волос</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,60 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex VI/12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 10 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,30 %</t>
-  </si>
-  <si>
     <t xml:space="preserve">Annex V/29</t>
   </si>
   <si>
     <t xml:space="preserve">Не более 1,0 %</t>
   </si>
   <si>
-    <t xml:space="preserve">0,50 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Diazolidinyl Urea</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex V/46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 0,5 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,24 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Methylparaben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex V/12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 0,4 % (как кислота)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,09 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Propylparaben</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex V/12a</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 0,14 % (сумма с бутилпарабеном)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,02 %</t>
+    <t xml:space="preserve">0,90 % (из Euxyl PE 9010)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сорбиновая кислота и её соли</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annex V/4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не более 0,6 % в пересчёте на кислоту</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potassium Sorbate 0,30 % ≈ 0,22 % кислоты</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethylhexylglycerin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не входит в Annex V, усилитель консервантов без ограничений</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,10 %</t>
   </si>
   <si>
     <t xml:space="preserve">Annex III/53</t>
@@ -807,7 +834,19 @@
     <t xml:space="preserve">0,03 %</t>
   </si>
   <si>
-    <t xml:space="preserve">Формальдегид (из Diazolidinyl Urea)</t>
+    <t xml:space="preserve">Парабены, Diazolidinyl Urea</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annex V/12, 12a, 46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разрешены с лимитами, но исключены из рецептуры</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Отсутствуют</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Формальдегид</t>
   </si>
   <si>
     <t xml:space="preserve">Регл. 2022/1181</t>
@@ -816,7 +855,7 @@
     <t xml:space="preserve">Надпись «выделяет формальдегид» при содержании более 0,001 %</t>
   </si>
   <si>
-    <t xml:space="preserve">Проверить аналитически; при 0,24 % DU надпись, скорее всего, потребуется</t>
+    <t xml:space="preserve">Не требуется: формальдегид-доноров нет</t>
   </si>
   <si>
     <t xml:space="preserve">Аллергены отдушки</t>
@@ -846,10 +885,10 @@
     <t xml:space="preserve">Ориентировочный INCI готового продукта (по убыванию; компоненты ниже 1 % можно указывать в любом порядке)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aqua, Isododecane, Glycerin, Dimethicone, Sorbitol, Propylene Glycol, C12-15 Alkyl Benzoate, Cetyl Alcohol, Behentrimonium Chloride, Phenyl Trimethicone, Betaine, Sodium PCA, Panthenol, Phenoxyethanol, PEG-40 Hydrogenated Castor Oil, Acetamidoethoxyethanol, Parfum, Ethylhexyl Methoxycinnamate, PEG-12 Dimethicone, Behentrimonium Methosulfate, Diazolidinyl Urea, Silicone Quaternium-18, Argania Spinosa Kernel Oil, Dimethiconol, Niacinamide, PEG/PPG-15/15 Dimethicone, C10-40 Isoalkylamidopropylethyldimonium Ethosulfate, Hydrolyzed Keratin, Lactic Acid, Tetrasodium EDTA, Caffeine, Gossypium Herbaceum (Cotton) Seed Oil, Methylparaben, Hydrolyzed Silk, Trideceth-6, Trideceth-12, Glycine Soja Protein, Oryza Sativa Extract, Triticum Vulgare (Wheat) Germ Extract, Etidronic Acid, Propylparaben, Sodium Hyaluronate, Carboxymethyl Chitin, [аллергены отдушки по декларации]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Порядок INCI уточняется после получения TDS на смесевое сырьё (доли компонентов в Cutissential Behenyl 18-MEA, Silsoft Q PMF, PMX-1503, Germaben II) и выбора грейда Behentrimonium Chloride (растворитель грейда добавить в INCI).</t>
+    <t xml:space="preserve">Aqua, Isododecane, Glycerin, Dimethicone, Phenoxyethanol, C12-15 Alkyl Benzoate, Sorbitol, Cetyl Alcohol, Behentrimonium Chloride, Propylene Glycol, Phenyl Trimethicone, Betaine, Sodium PCA, Panthenol, PEG-40 Hydrogenated Castor Oil, Acetamidoethoxyethanol, Behentrimonium Methosulfate, Parfum, Potassium Sorbate, Ethylhexyl Methoxycinnamate, PEG-12 Dimethicone, Silicone Quaternium-18, Argania Spinosa Kernel Oil, Dimethiconol, Niacinamide, PEG/PPG-15/15 Dimethicone, Lactic Acid, Hydrolyzed Keratin, Butylene Glycol, Ethylhexylglycerin, Tetrasodium EDTA, Caffeine, Gossypium Herbaceum (Cotton) Seed Oil, Hydrolyzed Silk, Trideceth-6, Trideceth-12, Glycine Soja Protein, Oryza Sativa Extract, Triticum Vulgare (Wheat) Germ Extract, Etidronic Acid, Sodium Hyaluronate, Carboxymethyl Chitin, [аллергены отдушки по декларации]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Порядок INCI уточняется после получения TDS на смесевое сырьё (доли компонентов в Incroquat Behenyl TMS-50, Silsoft Q PMF, PMX-1503, Euxyl PE 9010) и выбора грейда Behentrimonium Chloride (растворитель грейда добавить в INCI).</t>
   </si>
 </sst>
 </file>
@@ -1424,11 +1463,11 @@
       </c>
       <c r="F6" s="9" t="n">
         <f aca="false">100-SUM(F7:F47)</f>
-        <v>79.73</v>
+        <v>79.68</v>
       </c>
       <c r="G6" s="9" t="n">
         <f aca="false">F6*E6/100</f>
-        <v>79.73</v>
+        <v>79.68</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>15</v>
@@ -1551,9 +1590,7 @@
       <c r="H10" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="I10" s="7" t="s">
-        <v>30</v>
-      </c>
+      <c r="I10" s="7"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="n">
@@ -1563,10 +1600,10 @@
         <v>12</v>
       </c>
       <c r="C11" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="D11" s="7" t="s">
         <v>31</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>32</v>
       </c>
       <c r="E11" s="8" t="n">
         <v>100</v>
@@ -1579,7 +1616,7 @@
         <v>0.5</v>
       </c>
       <c r="H11" s="7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I11" s="7"/>
     </row>
@@ -1591,10 +1628,10 @@
         <v>12</v>
       </c>
       <c r="C12" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="7" t="s">
         <v>34</v>
-      </c>
-      <c r="D12" s="7" t="s">
-        <v>35</v>
       </c>
       <c r="E12" s="8" t="n">
         <v>100</v>
@@ -1607,10 +1644,10 @@
         <v>0.2</v>
       </c>
       <c r="H12" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="I12" s="7" t="s">
         <v>36</v>
-      </c>
-      <c r="I12" s="7" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1621,10 +1658,10 @@
         <v>12</v>
       </c>
       <c r="C13" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D13" s="7" t="s">
         <v>38</v>
-      </c>
-      <c r="D13" s="7" t="s">
-        <v>39</v>
       </c>
       <c r="E13" s="8" t="n">
         <v>100</v>
@@ -1637,10 +1674,10 @@
         <v>0.1</v>
       </c>
       <c r="H13" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="I13" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="I13" s="7" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1651,10 +1688,10 @@
         <v>12</v>
       </c>
       <c r="C14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D14" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>43</v>
       </c>
       <c r="E14" s="8" t="n">
         <v>100</v>
@@ -1667,15 +1704,15 @@
         <v>0.02</v>
       </c>
       <c r="H14" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="I14" s="7" t="s">
         <v>44</v>
-      </c>
-      <c r="I14" s="7" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B15" s="4"/>
       <c r="C15" s="4"/>
@@ -1691,13 +1728,13 @@
         <v>10</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="D16" s="7" t="s">
         <v>48</v>
-      </c>
-      <c r="D16" s="7" t="s">
-        <v>49</v>
       </c>
       <c r="E16" s="8" t="n">
         <v>80</v>
@@ -1710,70 +1747,70 @@
         <v>0.6</v>
       </c>
       <c r="H16" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="I16" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="I16" s="7" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="n">
         <v>11</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="D17" s="7" t="s">
         <v>52</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>53</v>
       </c>
       <c r="E17" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G17" s="9" t="n">
         <f aca="false">F17*E17/100</f>
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H17" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="I17" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="I17" s="7" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="n">
         <v>12</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C18" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="D18" s="7" t="s">
         <v>56</v>
-      </c>
-      <c r="D18" s="7" t="s">
-        <v>57</v>
       </c>
       <c r="E18" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="G18" s="9" t="n">
         <f aca="false">F18*E18/100</f>
-        <v>0.2</v>
+        <v>0.4</v>
       </c>
       <c r="H18" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="I18" s="7" t="s">
         <v>58</v>
-      </c>
-      <c r="I18" s="7" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1781,13 +1818,13 @@
         <v>13</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C19" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>60</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>61</v>
       </c>
       <c r="E19" s="8" t="n">
         <v>100</v>
@@ -1800,7 +1837,7 @@
         <v>0.8</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="I19" s="7"/>
     </row>
@@ -1809,13 +1846,13 @@
         <v>14</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C20" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>63</v>
-      </c>
-      <c r="D20" s="7" t="s">
-        <v>64</v>
       </c>
       <c r="E20" s="8" t="n">
         <v>100</v>
@@ -1828,10 +1865,10 @@
         <v>0.3</v>
       </c>
       <c r="H20" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="I20" s="7" t="s">
         <v>65</v>
-      </c>
-      <c r="I20" s="7" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1839,13 +1876,13 @@
         <v>15</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C21" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>68</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>100</v>
@@ -1858,7 +1895,7 @@
         <v>0.5</v>
       </c>
       <c r="H21" s="7" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="I21" s="7"/>
     </row>
@@ -1867,13 +1904,13 @@
         <v>16</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C22" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D22" s="7" t="s">
         <v>70</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>71</v>
       </c>
       <c r="E22" s="8" t="n">
         <v>100</v>
@@ -1886,10 +1923,10 @@
         <v>1.5</v>
       </c>
       <c r="H22" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="I22" s="7" t="s">
         <v>72</v>
-      </c>
-      <c r="I22" s="7" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1897,13 +1934,13 @@
         <v>17</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C23" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>74</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>75</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>100</v>
@@ -1916,7 +1953,7 @@
         <v>0.2</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I23" s="7"/>
     </row>
@@ -1925,13 +1962,13 @@
         <v>18</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C24" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>77</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>78</v>
       </c>
       <c r="E24" s="8" t="n">
         <v>100</v>
@@ -1944,7 +1981,7 @@
         <v>0.1</v>
       </c>
       <c r="H24" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="I24" s="7"/>
     </row>
@@ -1953,13 +1990,13 @@
         <v>19</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C25" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="D25" s="7" t="s">
         <v>80</v>
-      </c>
-      <c r="D25" s="7" t="s">
-        <v>81</v>
       </c>
       <c r="E25" s="8" t="n">
         <v>100</v>
@@ -1972,15 +2009,15 @@
         <v>0.2</v>
       </c>
       <c r="H25" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="I25" s="7" t="s">
         <v>82</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B26" s="4"/>
       <c r="C26" s="4"/>
@@ -1996,13 +2033,13 @@
         <v>20</v>
       </c>
       <c r="B27" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C27" s="6" t="s">
+      <c r="D27" s="7" t="s">
         <v>86</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>87</v>
       </c>
       <c r="E27" s="8" t="n">
         <v>100</v>
@@ -2015,15 +2052,15 @@
         <v>2.5</v>
       </c>
       <c r="H27" s="7" t="s">
+        <v>87</v>
+      </c>
+      <c r="I27" s="7" t="s">
         <v>88</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B28" s="4"/>
       <c r="C28" s="4"/>
@@ -2039,13 +2076,13 @@
         <v>21</v>
       </c>
       <c r="B29" s="5" t="s">
+        <v>90</v>
+      </c>
+      <c r="C29" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="D29" s="7" t="s">
         <v>92</v>
-      </c>
-      <c r="D29" s="7" t="s">
-        <v>93</v>
       </c>
       <c r="E29" s="8" t="n">
         <v>100</v>
@@ -2058,10 +2095,10 @@
         <v>1</v>
       </c>
       <c r="H29" s="7" t="s">
+        <v>93</v>
+      </c>
+      <c r="I29" s="7" t="s">
         <v>94</v>
-      </c>
-      <c r="I29" s="7" t="s">
-        <v>95</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2069,13 +2106,13 @@
         <v>22</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C30" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="D30" s="7" t="s">
-        <v>97</v>
       </c>
       <c r="E30" s="8" t="n">
         <v>100</v>
@@ -2088,7 +2125,7 @@
         <v>0.3</v>
       </c>
       <c r="H30" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="I30" s="7"/>
     </row>
@@ -2097,13 +2134,13 @@
         <v>23</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C31" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="D31" s="7" t="s">
         <v>99</v>
-      </c>
-      <c r="D31" s="7" t="s">
-        <v>100</v>
       </c>
       <c r="E31" s="8" t="n">
         <v>75</v>
@@ -2116,10 +2153,10 @@
         <v>0.525</v>
       </c>
       <c r="H31" s="7" t="s">
+        <v>100</v>
+      </c>
+      <c r="I31" s="7" t="s">
         <v>101</v>
-      </c>
-      <c r="I31" s="7" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2127,13 +2164,13 @@
         <v>24</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C32" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>103</v>
-      </c>
-      <c r="D32" s="7" t="s">
-        <v>104</v>
       </c>
       <c r="E32" s="8" t="n">
         <v>50</v>
@@ -2146,10 +2183,10 @@
         <v>0.5</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="I32" s="7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2157,13 +2194,13 @@
         <v>25</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C33" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>106</v>
-      </c>
-      <c r="D33" s="7" t="s">
-        <v>107</v>
       </c>
       <c r="E33" s="8" t="n">
         <v>100</v>
@@ -2176,7 +2213,7 @@
         <v>0.5</v>
       </c>
       <c r="H33" s="7" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="I33" s="7"/>
     </row>
@@ -2185,13 +2222,13 @@
         <v>26</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C34" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="D34" s="7" t="s">
         <v>109</v>
-      </c>
-      <c r="D34" s="7" t="s">
-        <v>110</v>
       </c>
       <c r="E34" s="8" t="n">
         <v>25</v>
@@ -2204,10 +2241,10 @@
         <v>0.125</v>
       </c>
       <c r="H34" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="I34" s="7" t="s">
         <v>111</v>
-      </c>
-      <c r="I34" s="7" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2215,13 +2252,13 @@
         <v>27</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C35" s="6" t="s">
+        <v>112</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>113</v>
-      </c>
-      <c r="D35" s="7" t="s">
-        <v>114</v>
       </c>
       <c r="E35" s="8" t="n">
         <v>25</v>
@@ -2234,7 +2271,7 @@
         <v>0.075</v>
       </c>
       <c r="H35" s="7" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="I35" s="7"/>
     </row>
@@ -2243,13 +2280,13 @@
         <v>28</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C36" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="D36" s="7" t="s">
         <v>116</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>117</v>
       </c>
       <c r="E36" s="8" t="n">
         <v>20</v>
@@ -2262,10 +2299,10 @@
         <v>0.04</v>
       </c>
       <c r="H36" s="7" t="s">
+        <v>117</v>
+      </c>
+      <c r="I36" s="7" t="s">
         <v>118</v>
-      </c>
-      <c r="I36" s="7" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2273,13 +2310,13 @@
         <v>29</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C37" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D37" s="7" t="s">
         <v>120</v>
-      </c>
-      <c r="D37" s="7" t="s">
-        <v>121</v>
       </c>
       <c r="E37" s="8" t="n">
         <v>100</v>
@@ -2292,10 +2329,10 @@
         <v>0.2</v>
       </c>
       <c r="H37" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="I37" s="7" t="s">
         <v>122</v>
-      </c>
-      <c r="I37" s="7" t="s">
-        <v>123</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2303,13 +2340,13 @@
         <v>30</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C38" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="D38" s="7" t="s">
         <v>124</v>
-      </c>
-      <c r="D38" s="7" t="s">
-        <v>125</v>
       </c>
       <c r="E38" s="8" t="n">
         <v>100</v>
@@ -2322,10 +2359,10 @@
         <v>0.2</v>
       </c>
       <c r="H38" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="I38" s="7" t="s">
         <v>126</v>
-      </c>
-      <c r="I38" s="7" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2333,13 +2370,13 @@
         <v>31</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C39" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="D39" s="7" t="s">
         <v>128</v>
-      </c>
-      <c r="D39" s="7" t="s">
-        <v>129</v>
       </c>
       <c r="E39" s="8" t="n">
         <v>1</v>
@@ -2352,10 +2389,10 @@
         <v>0.01</v>
       </c>
       <c r="H39" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="I39" s="7" t="s">
         <v>130</v>
-      </c>
-      <c r="I39" s="7" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2363,13 +2400,13 @@
         <v>32</v>
       </c>
       <c r="B40" s="5" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C40" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D40" s="7" t="s">
         <v>132</v>
-      </c>
-      <c r="D40" s="7" t="s">
-        <v>133</v>
       </c>
       <c r="E40" s="8" t="n">
         <v>60</v>
@@ -2382,15 +2419,15 @@
         <v>0.03</v>
       </c>
       <c r="H40" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="I40" s="7" t="s">
         <v>134</v>
-      </c>
-      <c r="I40" s="7" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B41" s="4"/>
       <c r="C41" s="4"/>
@@ -2401,64 +2438,64 @@
       <c r="H41" s="4"/>
       <c r="I41" s="4"/>
     </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="n">
         <v>33</v>
       </c>
       <c r="B42" s="5" t="s">
+        <v>136</v>
+      </c>
+      <c r="C42" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="C42" s="6" t="s">
+      <c r="D42" s="7" t="s">
         <v>138</v>
-      </c>
-      <c r="D42" s="7" t="s">
-        <v>139</v>
       </c>
       <c r="E42" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="G42" s="9" t="n">
         <f aca="false">F42*E42/100</f>
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="H42" s="7" t="s">
+        <v>139</v>
+      </c>
+      <c r="I42" s="7" t="s">
         <v>140</v>
       </c>
-      <c r="I42" s="7" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="n">
         <v>34</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C43" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="D43" s="7" t="s">
         <v>142</v>
-      </c>
-      <c r="D43" s="7" t="s">
-        <v>143</v>
       </c>
       <c r="E43" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="G43" s="9" t="n">
         <f aca="false">F43*E43/100</f>
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="H43" s="7" t="s">
+        <v>143</v>
+      </c>
+      <c r="I43" s="7" t="s">
         <v>144</v>
-      </c>
-      <c r="I43" s="7" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2466,13 +2503,13 @@
         <v>35</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C44" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D44" s="7" t="s">
         <v>146</v>
-      </c>
-      <c r="D44" s="7" t="s">
-        <v>147</v>
       </c>
       <c r="E44" s="8" t="n">
         <v>100</v>
@@ -2485,10 +2522,10 @@
         <v>0.5</v>
       </c>
       <c r="H44" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="I44" s="7" t="s">
         <v>148</v>
-      </c>
-      <c r="I44" s="7" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2496,13 +2533,13 @@
         <v>36</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C45" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D45" s="7" t="s">
         <v>150</v>
-      </c>
-      <c r="D45" s="7" t="s">
-        <v>151</v>
       </c>
       <c r="E45" s="8" t="n">
         <v>100</v>
@@ -2515,15 +2552,15 @@
         <v>0.4</v>
       </c>
       <c r="H45" s="7" t="s">
+        <v>151</v>
+      </c>
+      <c r="I45" s="7" t="s">
         <v>152</v>
-      </c>
-      <c r="I45" s="7" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B46" s="4"/>
       <c r="C46" s="4"/>
@@ -2539,36 +2576,36 @@
         <v>37</v>
       </c>
       <c r="B47" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="C47" s="6" t="s">
         <v>155</v>
       </c>
-      <c r="C47" s="6" t="s">
+      <c r="D47" s="7" t="s">
         <v>156</v>
-      </c>
-      <c r="D47" s="7" t="s">
-        <v>157</v>
       </c>
       <c r="E47" s="8" t="n">
         <v>80</v>
       </c>
       <c r="F47" s="10" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G47" s="9" t="n">
         <f aca="false">F47*E47/100</f>
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="H47" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="I47" s="7" t="s">
         <v>158</v>
-      </c>
-      <c r="I47" s="7" t="s">
-        <v>159</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11"/>
       <c r="B48" s="11"/>
       <c r="C48" s="12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D48" s="11"/>
       <c r="E48" s="11"/>
@@ -2582,7 +2619,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C50" s="14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2591,12 +2628,12 @@
       </c>
       <c r="F51" s="16" t="n">
         <f aca="false">SUM(F6:F14)</f>
-        <v>83.65</v>
+        <v>83.6</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C52" s="15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F52" s="16" t="n">
         <f aca="false">SUM(F16:F25)</f>
@@ -2605,7 +2642,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C53" s="15" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F53" s="16" t="n">
         <f aca="false">SUM(F27:F27)</f>
@@ -2614,7 +2651,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C54" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="F54" s="16" t="n">
         <f aca="false">SUM(F29:F40)</f>
@@ -2623,7 +2660,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C55" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F55" s="16" t="n">
         <f aca="false">SUM(F42:F45)</f>
@@ -2632,16 +2669,16 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C56" s="15" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="F56" s="16" t="n">
         <f aca="false">SUM(F47:F47)</f>
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C57" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F57" s="16" t="n">
         <f aca="false">SUM(F19:F25)+SUM(F27:F27)</f>
@@ -2650,7 +2687,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C58" s="15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F58" s="16" t="n">
         <f aca="false">SUM(F16:F18)</f>
@@ -2659,7 +2696,7 @@
     </row>
     <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C60" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -2694,7 +2731,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C27"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -2704,222 +2741,240 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>167</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
+        <v>168</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>169</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="C4" s="7" t="s">
         <v>170</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>172</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="7" t="s">
         <v>173</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>175</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="C6" s="7" t="s">
         <v>176</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>178</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="C7" s="7" t="s">
         <v>179</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>181</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="C8" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="C8" s="7" t="s">
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>184</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="C9" s="7" t="s">
         <v>185</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="6" t="s">
         <v>187</v>
       </c>
-      <c r="B10" s="6" t="s">
+      <c r="C10" s="7" t="s">
         <v>188</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3"/>
       <c r="B13" s="3" t="s">
+        <v>190</v>
+      </c>
+      <c r="C13" s="3" t="s">
         <v>191</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17"/>
       <c r="B14" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="C14" s="7" t="s">
         <v>193</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17"/>
       <c r="B15" s="6" t="s">
+        <v>194</v>
+      </c>
+      <c r="C15" s="7" t="s">
         <v>195</v>
-      </c>
-      <c r="C15" s="7" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17"/>
       <c r="B16" s="6" t="s">
+        <v>196</v>
+      </c>
+      <c r="C16" s="7" t="s">
         <v>197</v>
-      </c>
-      <c r="C16" s="7" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17"/>
       <c r="B17" s="6" t="s">
+        <v>198</v>
+      </c>
+      <c r="C17" s="7" t="s">
         <v>199</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>200</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17"/>
       <c r="B18" s="6" t="s">
+        <v>200</v>
+      </c>
+      <c r="C18" s="7" t="s">
         <v>201</v>
-      </c>
-      <c r="C18" s="7" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17"/>
       <c r="B19" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="C19" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="C19" s="7" t="s">
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="17"/>
+      <c r="B20" s="6" t="s">
         <v>204</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="s">
+      <c r="C20" s="7" t="s">
         <v>205</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3" t="s">
+      <c r="A22" s="14" t="s">
         <v>206</v>
       </c>
-      <c r="C22" s="3" t="s">
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3"/>
+      <c r="B23" s="3" t="s">
         <v>207</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="17"/>
-      <c r="B23" s="6" t="s">
+      <c r="C23" s="3" t="s">
         <v>208</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>209</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17"/>
       <c r="B24" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="C24" s="7" t="s">
         <v>210</v>
-      </c>
-      <c r="C24" s="7" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17"/>
       <c r="B25" s="6" t="s">
+        <v>211</v>
+      </c>
+      <c r="C25" s="7" t="s">
         <v>212</v>
-      </c>
-      <c r="C25" s="7" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17"/>
       <c r="B26" s="6" t="s">
+        <v>213</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="C26" s="7" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17"/>
       <c r="B27" s="6" t="s">
+        <v>215</v>
+      </c>
+      <c r="C27" s="7" t="s">
         <v>216</v>
       </c>
-      <c r="C27" s="7" t="s">
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="17"/>
+      <c r="B28" s="6" t="s">
         <v>217</v>
+      </c>
+      <c r="C28" s="7" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="17"/>
+      <c r="B29" s="6" t="s">
+        <v>219</v>
+      </c>
+      <c r="C29" s="7" t="s">
+        <v>220</v>
       </c>
     </row>
   </sheetData>
@@ -2938,7 +2993,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -2949,242 +3004,278 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B5" s="7" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="C6" s="7" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>227</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="s">
-        <v>228</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>229</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="14" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
-        <v>232</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>233</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>234</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>235</v>
+      <c r="C8" s="7" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>237</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>239</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>48</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>236</v>
-      </c>
-      <c r="C11" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="D11" s="7" t="s">
-        <v>238</v>
+      <c r="A11" s="14" t="s">
+        <v>240</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>239</v>
-      </c>
-      <c r="C12" s="7" t="s">
-        <v>240</v>
-      </c>
-      <c r="D12" s="7" t="s">
+      <c r="A12" s="3" t="s">
         <v>241</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>138</v>
+        <v>47</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>249</v>
+        <v>62</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>132</v>
+        <v>259</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>261</v>
+        <v>249</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>264</v>
+        <v>131</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="B20" s="7" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
         <v>272</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="18" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>273</v>
       </c>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-    </row>
-    <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="B21" s="7" t="s">
         <v>274</v>
       </c>
-      <c r="B25" s="2"/>
-      <c r="C25" s="2"/>
-      <c r="D25" s="2"/>
+      <c r="C21" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B22" s="7" t="s">
+        <v>278</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>279</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>282</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="14" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="18" t="s">
+        <v>286</v>
+      </c>
+      <c r="B26" s="18"/>
+      <c r="C26" s="18"/>
+      <c r="D26" s="18"/>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="A28:D28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Formulation v1.2: cationic pair on in-stock raw materials, no BTMS
- Drop the BTMS blend (Incroquat Behenyl TMS-50 is not available at the
  plant). Behentrimonium Chloride raised to 1.25% as supplied (1.0%
  active) and cetyl alcohol to 0.70%, keeping total cationics at 1.0%
  and fatty alcohol at ~0.7% as in v1.0/v1.1.
- Non-European sourcing notes: Quartamin AB (Kao), Chinese BTAC 80%,
  Asian cetyl alcohol; Samyang KCI BTMS 7550KC as the optional BTMS
  route; phenoxyethanol + ethylhexylglycerin dosed separately as the
  non-European alternative to Euxyl PE 9010.
- Position numbering, phase-sum labels, EU table and label INCI
  updated in xlsx, md and pdf.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UmFF3CgoK15mLAmmhMv9dF
</commit_message>
<xml_diff>
--- a/estel-18-plus/estel-18-plus-spray-formula.xlsx
+++ b/estel-18-plus/estel-18-plus-spray-formula.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="332" uniqueCount="288">
-  <si>
-    <t xml:space="preserve">Рецептура: несмываемый спрей-молочко для волос типа ESTEL 18 PLUS (рынок ЕС, без D5). Версия 1.1 от 08.10.2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Однородная белая эмульсия на катионных ПАВ, вязкость около 100 мПа·с, pH 4,8. Версия 1.1: комплекс 18-MEA заменён на Incroquat Behenyl TMS-50, Germaben II и феноксиэтанол заменены на Euxyl PE 9010 + сорбат калия. Дозировки: оценка по INCI оригинала и измерениям эталона (pH 5, плотность 1,01, вязкость около 100 мПа·с), требуют лабораторной проверки. Синим выделены вводимые значения (дозировки, активность сырья), чёрным: формулы.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="281">
+  <si>
+    <t xml:space="preserve">Рецептура: несмываемый спрей-молочко для волос типа ESTEL 18 PLUS (рынок ЕС, без D5). Версия 1.2 от 08.10.2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Однородная белая эмульсия на катионных ПАВ, вязкость около 100 мПа·с, pH 4,8. Версия 1.2: комплекс 18-MEA убран, катионная пара собрана на Behentrimonium Chloride и цетиловом спирте; Germaben II и феноксиэтанол заменены на Euxyl PE 9010 + сорбат калия. Дозировки: оценка по INCI оригинала и измерениям эталона (pH 5, плотность 1,01, вязкость около 100 мПа·с), требуют лабораторной проверки. Синим выделены вводимые значения (дозировки, активность сырья), чёрным: формулы.</t>
   </si>
   <si>
     <t xml:space="preserve">№</t>
@@ -171,37 +171,25 @@
     <t xml:space="preserve">Behentrimonium Chloride</t>
   </si>
   <si>
-    <t xml:space="preserve">Genamin KDMP (Clariant) / Incroquat Behenyl TMC-85 (Croda, 85 %) / Varisoft BT 85 Pellets (Evonik); гранулы ~80 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Катионный эмульгатор, кондиционер, антистатик, термозащита</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,6 % активного. Растворитель грейда (изопропанол или этанол) указать в INCI. ЕС Annex III/287: не более 3 % в несмываемых средствах для волос</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Behentrimonium Methosulfate (and) Cetyl Alcohol (and) Butylene Glycol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Incroquat Behenyl TMS-50 (Croda); аналоги: BTMS-50 других поставщиков с тем же INCI</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Катионный эмульгатор и кондиционер, структурообразователь (замена комплекса 18-MEA)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ориентировочно 50 % BTMS, ~37 % цетилового спирта, ~13 % бутиленгликоля (уточнить по TDS). Даёт 0,4 % BTMS и ~0,3 % цетилового спирта. Не заменять на BTMS-25 (Varisoft BT 85, Incroquat Behenyl TMS): там цетеариловый спирт, вязкость вырастет, INCI изменится</t>
+    <t xml:space="preserve">Гранулы ~80 %: Genamin KDMP (Clariant), Incroquat Behenyl TMC-85 (Croda, 85 %), Varisoft BT 85 Pellets (Evonik); не европейские: Quartamin AB (Kao, Япония), Behentrimonium Chloride 80 % китайских производителей (напр., Suzhou Wedo Chemicals)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Единственный катионный эмульгатор: кондиционер, антистатик, термозащита; с цетиловым спиртом даёт структуру эмульсии</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1,0 % активного: столько же квата, сколько давали BTAC + BTMS в версиях 1.0 и 1.1. Растворитель грейда (изопропанол или этанол) указать в INCI. ЕС Annex III/287: не более 3 % в несмываемых средствах для волос. Если нужна мягкость метосульфата: не европейский BTMS-50 с INCI Behentrimonium Methosulfate, Cetyl Alcohol, Butylene Glycol, напр. Samyang KCI BTMS 7550KC (Корея): 0,8 % при BTAC 0,75 % и цетиловом спирте 0,4 %</t>
   </si>
   <si>
     <t xml:space="preserve">Cetyl Alcohol</t>
   </si>
   <si>
-    <t xml:space="preserve">Lanette 16 (BASF) / Crodacol C90 (Croda) / TEGO Alkanol 16 (Evonik)</t>
+    <t xml:space="preserve">Lanette 16 (BASF) / Crodacol C90 (Croda) / TEGO Alkanol 16 (Evonik); не европейские: цетиловый спирт 98 % азиатских олеохимических производителей (Малайзия, Индонезия, напр. KLK Oleo)</t>
   </si>
   <si>
     <t xml:space="preserve">Структурообразователь, регулятор вязкости</t>
   </si>
   <si>
-    <t xml:space="preserve">0,4 % компенсирует меньшую долю жирного спирта в TMS-50 по сравнению с комплексом 18-MEA; итого жирного спирта ~0,7 %. Диапазон 0,2–0,6 %: больше спирта, выше вязкость</t>
+    <t xml:space="preserve">0,7 %: весь жирный спирт теперь отдельным сырьём, раньше ~0,6 % приходило со смесевыми комплексами. Диапазон 0,5–0,9 %: больше спирта, выше вязкость</t>
   </si>
   <si>
     <t xml:space="preserve">C12-15 Alkyl Benzoate</t>
@@ -441,7 +429,7 @@
     <t xml:space="preserve">Phenoxyethanol (and) Ethylhexylglycerin</t>
   </si>
   <si>
-    <t xml:space="preserve">Euxyl PE 9010 (Schülke): феноксиэтанол 90 % + этилгексилглицерин 10 %</t>
+    <t xml:space="preserve">Euxyl PE 9010 (Schülke): феноксиэтанол 90 % + этилгексилглицерин 10 %; не европейский вариант: Phenoxyethanol 0,9 % + Ethylhexylglycerin 0,1 % по отдельности, любых производителей (Китай, Индия)</t>
   </si>
   <si>
     <t xml:space="preserve">Консервант широкого спектра с усилителем (замена феноксиэтанола 0,5 % и Germaben II 0,8 %)</t>
@@ -510,13 +498,13 @@
     <t xml:space="preserve">Сумма по фазам, % масс.</t>
   </si>
   <si>
-    <t xml:space="preserve">Масляная фаза без эмульгаторов (поз. 13–20)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Катионные ПАВ и цетиловый спирт, по сырью (поз. 10–12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Источники по сырью: Croda (Incroquat Behenyl TMS-50), Momentive (Silsoft Q PMF), Dow (XIAMETER PMX-1503, OFX-0193, DOWSIL 556), Nouryon (ElfaMoist AC), Schülke (Euxyl PE 9010); составы по TDS поставщиков. Параметры эталона: измерения технолога-заказчика.</t>
+    <t xml:space="preserve">Масляная фаза без эмульгаторов (поз. 12–19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Катионные ПАВ и цетиловый спирт, по сырью (поз. 10–11)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Источники по сырью: Momentive (Silsoft Q PMF), Dow (XIAMETER PMX-1503, OFX-0193, DOWSIL 556), Nouryon (ElfaMoist AC), Schülke (Euxyl PE 9010); составы по TDS поставщиков. Параметры эталона: измерения технолога-заказчика.</t>
   </si>
   <si>
     <t xml:space="preserve">Порядок изготовления (лабораторный замес, роторно-статорный гомогенизатор)</t>
@@ -669,7 +657,7 @@
     <t xml:space="preserve">Отстой масла или сливки</t>
   </si>
   <si>
-    <t xml:space="preserve">Усилить гомогенизацию на стадии 3; Incroquat Behenyl TMS-50 до 1,2 %</t>
+    <t xml:space="preserve">Усилить гомогенизацию на стадии 3; Behentrimonium Chloride до 1,5 % по сырью</t>
   </si>
   <si>
     <t xml:space="preserve">Помутнение, осадок</t>
@@ -720,7 +708,7 @@
     <t xml:space="preserve">Заменён</t>
   </si>
   <si>
-    <t xml:space="preserve">Incroquat Behenyl TMS-50 (Behentrimonium Methosulfate, Cetyl Alcohol, Butylene Glycol) 0,8 % плюс цетиловый спирт 0,4 %. Та же функциональная пара «бегениловый кват + цетиловый спирт», но без специального 18-MEA-квата: суммарно катионных ПАВ 1,0 % активного и жирного спирта ~0,7 %, как в версии 1.0, поэтому вязкость и кондиционирование сохраняются. Уходит только заявление о восстановлении липида 18-MEA. В INCI: минус C10-40 кват, плюс Butylene Glycol.</t>
+    <t xml:space="preserve">Версия 1.2: без нового смесевого сырья. Катионная пара собрана из уже имеющегося: Behentrimonium Chloride 1,25 % по сырью (1,0 % активного) плюс цетиловый спирт 0,7 %. Сумма катионных ПАВ 1,0 % и жирного спирта ~0,7 % те же, что в версиях 1.0 и 1.1, поэтому вязкость, стабильность эмульсии и кондиционирование сохраняются; уходит заявление о липиде 18-MEA. В INCI: минус C10-40 кват и Behentrimonium Methosulfate, новых компонентов нет. Если нужна мягкость метосульфата: не европейский BTMS-50 с INCI Behentrimonium Methosulfate, Cetyl Alcohol, Butylene Glycol (Samyang KCI BTMS 7550KC, Корея) 0,8 % при BTAC 0,75 % и цетиловом спирте 0,4 %. У китайских «BTMS-50» часто цетеариловый спирт: проверять INCI по COA.</t>
   </si>
   <si>
     <t xml:space="preserve">Germaben II (Propylene Glycol, Diazolidinyl Urea, Methylparaben, Propylparaben) и Phenoxyethanol 0,5 %</t>
@@ -768,57 +756,48 @@
     <t xml:space="preserve">Не более 3 % в несмываемых средствах для волос</t>
   </si>
   <si>
-    <t xml:space="preserve">0,60 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Behentrimonium Methosulfate</t>
+    <t xml:space="preserve">1,00 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annex VI/12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не более 10 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,30 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Phenoxyethanol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annex V/29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не более 1,0 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0,90 % (из Euxyl PE 9010)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сорбиновая кислота и её соли</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annex V/4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не более 0,6 % в пересчёте на кислоту</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Potassium Sorbate 0,30 % ≈ 0,22 % кислоты</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ethylhexylglycerin</t>
   </si>
   <si>
     <t xml:space="preserve">Не нормируется</t>
   </si>
   <si>
-    <t xml:space="preserve">Ограничений в приложениях Регл. 1223/2009 нет</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,40 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex VI/12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 10 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,30 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phenoxyethanol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex V/29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 1,0 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0,90 % (из Euxyl PE 9010)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сорбиновая кислота и её соли</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Annex V/4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Не более 0,6 % в пересчёте на кислоту</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Potassium Sorbate 0,30 % ≈ 0,22 % кислоты</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ethylhexylglycerin</t>
-  </si>
-  <si>
     <t xml:space="preserve">Не входит в Annex V, усилитель консервантов без ограничений</t>
   </si>
   <si>
@@ -885,10 +864,10 @@
     <t xml:space="preserve">Ориентировочный INCI готового продукта (по убыванию; компоненты ниже 1 % можно указывать в любом порядке)</t>
   </si>
   <si>
-    <t xml:space="preserve">Aqua, Isododecane, Glycerin, Dimethicone, Phenoxyethanol, C12-15 Alkyl Benzoate, Sorbitol, Cetyl Alcohol, Behentrimonium Chloride, Propylene Glycol, Phenyl Trimethicone, Betaine, Sodium PCA, Panthenol, PEG-40 Hydrogenated Castor Oil, Acetamidoethoxyethanol, Behentrimonium Methosulfate, Parfum, Potassium Sorbate, Ethylhexyl Methoxycinnamate, PEG-12 Dimethicone, Silicone Quaternium-18, Argania Spinosa Kernel Oil, Dimethiconol, Niacinamide, PEG/PPG-15/15 Dimethicone, Lactic Acid, Hydrolyzed Keratin, Butylene Glycol, Ethylhexylglycerin, Tetrasodium EDTA, Caffeine, Gossypium Herbaceum (Cotton) Seed Oil, Hydrolyzed Silk, Trideceth-6, Trideceth-12, Glycine Soja Protein, Oryza Sativa Extract, Triticum Vulgare (Wheat) Germ Extract, Etidronic Acid, Sodium Hyaluronate, Carboxymethyl Chitin, [аллергены отдушки по декларации]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Порядок INCI уточняется после получения TDS на смесевое сырьё (доли компонентов в Incroquat Behenyl TMS-50, Silsoft Q PMF, PMX-1503, Euxyl PE 9010) и выбора грейда Behentrimonium Chloride (растворитель грейда добавить в INCI).</t>
+    <t xml:space="preserve">Aqua, Isododecane, Glycerin, Dimethicone, Behentrimonium Chloride, Phenoxyethanol, C12-15 Alkyl Benzoate, Sorbitol, Cetyl Alcohol, Propylene Glycol, Phenyl Trimethicone, Betaine, Sodium PCA, Panthenol, PEG-40 Hydrogenated Castor Oil, Acetamidoethoxyethanol, Parfum, Potassium Sorbate, Ethylhexyl Methoxycinnamate, PEG-12 Dimethicone, Silicone Quaternium-18, Argania Spinosa Kernel Oil, Dimethiconol, Niacinamide, PEG/PPG-15/15 Dimethicone, Lactic Acid, Hydrolyzed Keratin, Ethylhexylglycerin, Tetrasodium EDTA, Caffeine, Gossypium Herbaceum (Cotton) Seed Oil, Hydrolyzed Silk, Trideceth-6, Trideceth-12, Glycine Soja Protein, Oryza Sativa Extract, Triticum Vulgare (Wheat) Germ Extract, Etidronic Acid, Sodium Hyaluronate, Carboxymethyl Chitin, [растворитель грейда Behentrimonium Chloride], [аллергены отдушки по декларации]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Порядок INCI уточняется после получения TDS на смесевое сырьё (доли компонентов в Silsoft Q PMF, PMX-1503) и выбора грейда Behentrimonium Chloride (растворитель грейда добавить в INCI).</t>
   </si>
 </sst>
 </file>
@@ -1371,7 +1350,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1462,7 +1441,7 @@
         <v>100</v>
       </c>
       <c r="F6" s="9" t="n">
-        <f aca="false">100-SUM(F7:F47)</f>
+        <f aca="false">100-SUM(F7:F46)</f>
         <v>79.68</v>
       </c>
       <c r="G6" s="9" t="n">
@@ -1723,7 +1702,7 @@
       <c r="H15" s="4"/>
       <c r="I15" s="4"/>
     </row>
-    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="n">
         <v>10</v>
       </c>
@@ -1740,11 +1719,11 @@
         <v>80</v>
       </c>
       <c r="F16" s="10" t="n">
-        <v>0.75</v>
+        <v>1.25</v>
       </c>
       <c r="G16" s="9" t="n">
         <f aca="false">F16*E16/100</f>
-        <v>0.6</v>
+        <v>1</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>49</v>
@@ -1770,11 +1749,11 @@
         <v>100</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="G17" s="9" t="n">
         <f aca="false">F17*E17/100</f>
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>53</v>
@@ -1783,7 +1762,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="n">
         <v>12</v>
       </c>
@@ -1800,18 +1779,16 @@
         <v>100</v>
       </c>
       <c r="F18" s="10" t="n">
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="G18" s="9" t="n">
         <f aca="false">F18*E18/100</f>
-        <v>0.4</v>
+        <v>0.8</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="I18" s="7" t="s">
-        <v>58</v>
-      </c>
+      <c r="I18" s="7"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="n">
@@ -1821,25 +1798,27 @@
         <v>46</v>
       </c>
       <c r="C19" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="7" t="s">
         <v>59</v>
-      </c>
-      <c r="D19" s="7" t="s">
-        <v>60</v>
       </c>
       <c r="E19" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F19" s="10" t="n">
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="G19" s="9" t="n">
         <f aca="false">F19*E19/100</f>
-        <v>0.8</v>
+        <v>0.3</v>
       </c>
       <c r="H19" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="I19" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="I19" s="7"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="n">
@@ -1858,20 +1837,18 @@
         <v>100</v>
       </c>
       <c r="F20" s="10" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="G20" s="9" t="n">
         <f aca="false">F20*E20/100</f>
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="H20" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="I20" s="7" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I20" s="7"/>
+    </row>
+    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="n">
         <v>15</v>
       </c>
@@ -1879,27 +1856,29 @@
         <v>46</v>
       </c>
       <c r="C21" s="6" t="s">
+        <v>65</v>
+      </c>
+      <c r="D21" s="7" t="s">
         <v>66</v>
-      </c>
-      <c r="D21" s="7" t="s">
-        <v>67</v>
       </c>
       <c r="E21" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F21" s="10" t="n">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="G21" s="9" t="n">
         <f aca="false">F21*E21/100</f>
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="H21" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="I21" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="I21" s="7"/>
-    </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="n">
         <v>16</v>
       </c>
@@ -1916,20 +1895,18 @@
         <v>100</v>
       </c>
       <c r="F22" s="10" t="n">
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="G22" s="9" t="n">
         <f aca="false">F22*E22/100</f>
-        <v>1.5</v>
+        <v>0.2</v>
       </c>
       <c r="H22" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="I22" s="7" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I22" s="7"/>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="n">
         <v>17</v>
       </c>
@@ -1937,27 +1914,27 @@
         <v>46</v>
       </c>
       <c r="C23" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D23" s="7" t="s">
         <v>73</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>74</v>
       </c>
       <c r="E23" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F23" s="10" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G23" s="9" t="n">
         <f aca="false">F23*E23/100</f>
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I23" s="7"/>
     </row>
-    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="n">
         <v>18</v>
       </c>
@@ -1965,118 +1942,120 @@
         <v>46</v>
       </c>
       <c r="C24" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="D24" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="D24" s="7" t="s">
-        <v>77</v>
       </c>
       <c r="E24" s="8" t="n">
         <v>100</v>
       </c>
       <c r="F24" s="10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G24" s="9" t="n">
         <f aca="false">F24*E24/100</f>
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="H24" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="I24" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="I24" s="7"/>
-    </row>
-    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="5" t="n">
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
+      <c r="I25" s="4"/>
+    </row>
+    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="5" t="n">
         <v>19</v>
       </c>
-      <c r="B25" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="D25" s="7" t="s">
+      <c r="B26" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="E25" s="8" t="n">
+      <c r="C26" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="D26" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="E26" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="F25" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G25" s="9" t="n">
-        <f aca="false">F25*E25/100</f>
-        <v>0.2</v>
-      </c>
-      <c r="H25" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="I25" s="7" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="4" t="s">
+      <c r="F26" s="10" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G26" s="9" t="n">
+        <f aca="false">F26*E26/100</f>
+        <v>2.5</v>
+      </c>
+      <c r="H26" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="B26" s="4"/>
-      <c r="C26" s="4"/>
-      <c r="D26" s="4"/>
-      <c r="E26" s="4"/>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-    </row>
-    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="n">
+      <c r="I26" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
+      <c r="I27" s="4"/>
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="5" t="n">
         <v>20</v>
       </c>
-      <c r="B27" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="D27" s="7" t="s">
+      <c r="B28" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="E27" s="8" t="n">
+      <c r="C28" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D28" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E28" s="8" t="n">
         <v>100</v>
       </c>
-      <c r="F27" s="10" t="n">
-        <v>2.5</v>
-      </c>
-      <c r="G27" s="9" t="n">
-        <f aca="false">F27*E27/100</f>
-        <v>2.5</v>
-      </c>
-      <c r="H27" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="I27" s="7" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="4" t="s">
+      <c r="F28" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="9" t="n">
+        <f aca="false">F28*E28/100</f>
+        <v>1</v>
+      </c>
+      <c r="H28" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="B28" s="4"/>
-      <c r="C28" s="4"/>
-      <c r="D28" s="4"/>
-      <c r="E28" s="4"/>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
+      <c r="I28" s="7" t="s">
+        <v>90</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="n">
         <v>21</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C29" s="6" t="s">
         <v>91</v>
@@ -2088,53 +2067,53 @@
         <v>100</v>
       </c>
       <c r="F29" s="10" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G29" s="9" t="n">
         <f aca="false">F29*E29/100</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="I29" s="7" t="s">
-        <v>94</v>
-      </c>
+      <c r="I29" s="7"/>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="n">
         <v>22</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C30" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="D30" s="7" t="s">
         <v>95</v>
       </c>
-      <c r="D30" s="7" t="s">
-        <v>96</v>
-      </c>
       <c r="E30" s="8" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="F30" s="10" t="n">
-        <v>0.3</v>
+        <v>0.7</v>
       </c>
       <c r="G30" s="9" t="n">
         <f aca="false">F30*E30/100</f>
-        <v>0.3</v>
+        <v>0.525</v>
       </c>
       <c r="H30" s="7" t="s">
+        <v>96</v>
+      </c>
+      <c r="I30" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="I30" s="7"/>
-    </row>
-    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="n">
         <v>23</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C31" s="6" t="s">
         <v>98</v>
@@ -2143,20 +2122,20 @@
         <v>99</v>
       </c>
       <c r="E31" s="8" t="n">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="F31" s="10" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="G31" s="9" t="n">
         <f aca="false">F31*E31/100</f>
-        <v>0.525</v>
+        <v>0.5</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>100</v>
       </c>
       <c r="I31" s="7" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2164,65 +2143,65 @@
         <v>24</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C32" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="D32" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="D32" s="7" t="s">
-        <v>103</v>
-      </c>
       <c r="E32" s="8" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="F32" s="10" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="G32" s="9" t="n">
         <f aca="false">F32*E32/100</f>
         <v>0.5</v>
       </c>
       <c r="H32" s="7" t="s">
-        <v>104</v>
-      </c>
-      <c r="I32" s="7" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>103</v>
+      </c>
+      <c r="I32" s="7"/>
+    </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="n">
         <v>25</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C33" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="D33" s="7" t="s">
         <v>105</v>
       </c>
-      <c r="D33" s="7" t="s">
-        <v>106</v>
-      </c>
       <c r="E33" s="8" t="n">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="F33" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="G33" s="9" t="n">
         <f aca="false">F33*E33/100</f>
-        <v>0.5</v>
+        <v>0.125</v>
       </c>
       <c r="H33" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="I33" s="7" t="s">
         <v>107</v>
       </c>
-      <c r="I33" s="7"/>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="n">
         <v>26</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C34" s="6" t="s">
         <v>108</v>
@@ -2234,53 +2213,53 @@
         <v>25</v>
       </c>
       <c r="F34" s="10" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="G34" s="9" t="n">
         <f aca="false">F34*E34/100</f>
-        <v>0.125</v>
+        <v>0.075</v>
       </c>
       <c r="H34" s="7" t="s">
         <v>110</v>
       </c>
-      <c r="I34" s="7" t="s">
-        <v>111</v>
-      </c>
+      <c r="I34" s="7"/>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="n">
         <v>27</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C35" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="D35" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D35" s="7" t="s">
-        <v>113</v>
-      </c>
       <c r="E35" s="8" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F35" s="10" t="n">
-        <v>0.3</v>
+        <v>0.2</v>
       </c>
       <c r="G35" s="9" t="n">
         <f aca="false">F35*E35/100</f>
-        <v>0.075</v>
+        <v>0.04</v>
       </c>
       <c r="H35" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="I35" s="7" t="s">
         <v>114</v>
       </c>
-      <c r="I35" s="7"/>
-    </row>
-    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="n">
         <v>28</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C36" s="6" t="s">
         <v>115</v>
@@ -2289,14 +2268,14 @@
         <v>116</v>
       </c>
       <c r="E36" s="8" t="n">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="F36" s="10" t="n">
         <v>0.2</v>
       </c>
       <c r="G36" s="9" t="n">
         <f aca="false">F36*E36/100</f>
-        <v>0.04</v>
+        <v>0.2</v>
       </c>
       <c r="H36" s="7" t="s">
         <v>117</v>
@@ -2305,12 +2284,12 @@
         <v>118</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="5" t="n">
         <v>29</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C37" s="6" t="s">
         <v>119</v>
@@ -2335,12 +2314,12 @@
         <v>122</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="n">
         <v>30</v>
       </c>
       <c r="B38" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C38" s="6" t="s">
         <v>123</v>
@@ -2349,14 +2328,14 @@
         <v>124</v>
       </c>
       <c r="E38" s="8" t="n">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="F38" s="10" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="G38" s="9" t="n">
         <f aca="false">F38*E38/100</f>
-        <v>0.2</v>
+        <v>0.01</v>
       </c>
       <c r="H38" s="7" t="s">
         <v>125</v>
@@ -2365,12 +2344,12 @@
         <v>126</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="n">
         <v>31</v>
       </c>
       <c r="B39" s="5" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C39" s="6" t="s">
         <v>127</v>
@@ -2379,14 +2358,14 @@
         <v>128</v>
       </c>
       <c r="E39" s="8" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F39" s="10" t="n">
-        <v>1</v>
+        <v>0.05</v>
       </c>
       <c r="G39" s="9" t="n">
         <f aca="false">F39*E39/100</f>
-        <v>0.01</v>
+        <v>0.03</v>
       </c>
       <c r="H39" s="7" t="s">
         <v>129</v>
@@ -2395,55 +2374,55 @@
         <v>130</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="n">
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B40" s="4"/>
+      <c r="C40" s="4"/>
+      <c r="D40" s="4"/>
+      <c r="E40" s="4"/>
+      <c r="F40" s="4"/>
+      <c r="G40" s="4"/>
+      <c r="H40" s="4"/>
+      <c r="I40" s="4"/>
+    </row>
+    <row r="41" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="n">
         <v>32</v>
       </c>
-      <c r="B40" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="C40" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D40" s="7" t="s">
+      <c r="B41" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="E40" s="8" t="n">
-        <v>60</v>
-      </c>
-      <c r="F40" s="10" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="G40" s="9" t="n">
-        <f aca="false">F40*E40/100</f>
-        <v>0.03</v>
-      </c>
-      <c r="H40" s="7" t="s">
+      <c r="C41" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="I40" s="7" t="s">
+      <c r="D41" s="7" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
+      <c r="E41" s="8" t="n">
+        <v>100</v>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="9" t="n">
+        <f aca="false">F41*E41/100</f>
+        <v>1</v>
+      </c>
+      <c r="H41" s="7" t="s">
         <v>135</v>
       </c>
-      <c r="B41" s="4"/>
-      <c r="C41" s="4"/>
-      <c r="D41" s="4"/>
-      <c r="E41" s="4"/>
-      <c r="F41" s="4"/>
-      <c r="G41" s="4"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-    </row>
-    <row r="42" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I41" s="7" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="n">
         <v>33</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C42" s="6" t="s">
         <v>137</v>
@@ -2455,11 +2434,11 @@
         <v>100</v>
       </c>
       <c r="F42" s="10" t="n">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G42" s="9" t="n">
         <f aca="false">F42*E42/100</f>
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="H42" s="7" t="s">
         <v>139</v>
@@ -2468,12 +2447,12 @@
         <v>140</v>
       </c>
     </row>
-    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="n">
         <v>34</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C43" s="6" t="s">
         <v>141</v>
@@ -2485,11 +2464,11 @@
         <v>100</v>
       </c>
       <c r="F43" s="10" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="G43" s="9" t="n">
         <f aca="false">F43*E43/100</f>
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="H43" s="7" t="s">
         <v>143</v>
@@ -2498,12 +2477,12 @@
         <v>144</v>
       </c>
     </row>
-    <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="n">
         <v>35</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="C44" s="6" t="s">
         <v>145</v>
@@ -2515,11 +2494,11 @@
         <v>100</v>
       </c>
       <c r="F44" s="10" t="n">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="G44" s="9" t="n">
         <f aca="false">F44*E44/100</f>
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="H44" s="7" t="s">
         <v>147</v>
@@ -2528,193 +2507,163 @@
         <v>148</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="n">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="B45" s="4"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="4"/>
+      <c r="F45" s="4"/>
+      <c r="G45" s="4"/>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4"/>
+    </row>
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="n">
         <v>36</v>
       </c>
-      <c r="B45" s="5" t="s">
-        <v>136</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="D45" s="7" t="s">
+      <c r="B46" s="5" t="s">
         <v>150</v>
       </c>
-      <c r="E45" s="8" t="n">
+      <c r="C46" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="D46" s="7" t="s">
+        <v>152</v>
+      </c>
+      <c r="E46" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="F46" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="G46" s="9" t="n">
+        <f aca="false">F46*E46/100</f>
+        <v>0.16</v>
+      </c>
+      <c r="H46" s="7" t="s">
+        <v>153</v>
+      </c>
+      <c r="I46" s="7" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="11"/>
+      <c r="B47" s="11"/>
+      <c r="C47" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="D47" s="11"/>
+      <c r="E47" s="11"/>
+      <c r="F47" s="13" t="n">
+        <f aca="false">SUM(F5:F46)</f>
         <v>100</v>
       </c>
-      <c r="F45" s="10" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G45" s="9" t="n">
-        <f aca="false">F45*E45/100</f>
-        <v>0.4</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>151</v>
-      </c>
-      <c r="I45" s="7" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="B46" s="4"/>
-      <c r="C46" s="4"/>
-      <c r="D46" s="4"/>
-      <c r="E46" s="4"/>
-      <c r="F46" s="4"/>
-      <c r="G46" s="4"/>
-      <c r="H46" s="4"/>
-      <c r="I46" s="4"/>
-    </row>
-    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="n">
-        <v>37</v>
-      </c>
-      <c r="B47" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="C47" s="6" t="s">
-        <v>155</v>
-      </c>
-      <c r="D47" s="7" t="s">
+      <c r="G47" s="11"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C49" s="14" t="s">
         <v>156</v>
       </c>
-      <c r="E47" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="F47" s="10" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="G47" s="9" t="n">
-        <f aca="false">F47*E47/100</f>
-        <v>0.16</v>
-      </c>
-      <c r="H47" s="7" t="s">
-        <v>157</v>
-      </c>
-      <c r="I47" s="7" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="11"/>
-      <c r="B48" s="11"/>
-      <c r="C48" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="D48" s="11"/>
-      <c r="E48" s="11"/>
-      <c r="F48" s="13" t="n">
-        <f aca="false">SUM(F5:F47)</f>
-        <v>100</v>
-      </c>
-      <c r="G48" s="11"/>
-      <c r="H48" s="11"/>
-      <c r="I48" s="11"/>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C50" s="14" t="s">
-        <v>160</v>
+      <c r="C50" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="F50" s="16" t="n">
+        <f aca="false">SUM(F6:F14)</f>
+        <v>83.6</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C51" s="15" t="s">
-        <v>11</v>
+        <v>45</v>
       </c>
       <c r="F51" s="16" t="n">
-        <f aca="false">SUM(F6:F14)</f>
-        <v>83.6</v>
+        <f aca="false">SUM(F16:F24)</f>
+        <v>5.55</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C52" s="15" t="s">
-        <v>45</v>
+        <v>79</v>
       </c>
       <c r="F52" s="16" t="n">
-        <f aca="false">SUM(F16:F25)</f>
-        <v>5.55</v>
+        <f aca="false">SUM(F26:F26)</f>
+        <v>2.5</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C53" s="15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F53" s="16" t="n">
-        <f aca="false">SUM(F27:F27)</f>
-        <v>2.5</v>
+        <f aca="false">SUM(F28:F39)</f>
+        <v>5.95</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C54" s="15" t="s">
-        <v>89</v>
+        <v>131</v>
       </c>
       <c r="F54" s="16" t="n">
-        <f aca="false">SUM(F29:F40)</f>
-        <v>5.95</v>
+        <f aca="false">SUM(F41:F44)</f>
+        <v>2.2</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C55" s="15" t="s">
-        <v>135</v>
+        <v>149</v>
       </c>
       <c r="F55" s="16" t="n">
-        <f aca="false">SUM(F42:F45)</f>
-        <v>2.2</v>
+        <f aca="false">SUM(F46:F46)</f>
+        <v>0.2</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C56" s="15" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="F56" s="16" t="n">
-        <f aca="false">SUM(F47:F47)</f>
-        <v>0.2</v>
+        <f aca="false">SUM(F18:F24)+SUM(F26:F26)</f>
+        <v>6.1</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C57" s="15" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="F57" s="16" t="n">
-        <f aca="false">SUM(F19:F25)+SUM(F27:F27)</f>
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C58" s="15" t="s">
-        <v>162</v>
-      </c>
-      <c r="F58" s="16" t="n">
-        <f aca="false">SUM(F16:F18)</f>
+        <f aca="false">SUM(F16:F17)</f>
         <v>1.95</v>
       </c>
     </row>
-    <row r="60" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C60" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-      <c r="G60" s="2"/>
-      <c r="H60" s="2"/>
-      <c r="I60" s="2"/>
+    <row r="59" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C59" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+      <c r="G59" s="2"/>
+      <c r="H59" s="2"/>
+      <c r="I59" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="A2:I2"/>
     <mergeCell ref="A5:I5"/>
     <mergeCell ref="A15:I15"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A28:I28"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A46:I46"/>
-    <mergeCell ref="C60:I60"/>
+    <mergeCell ref="A25:I25"/>
+    <mergeCell ref="A27:I27"/>
+    <mergeCell ref="A40:I40"/>
+    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="C59:I59"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2741,240 +2690,240 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>166</v>
+        <v>162</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3"/>
       <c r="B13" s="3" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17"/>
       <c r="B14" s="6" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17"/>
       <c r="B15" s="6" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17"/>
       <c r="B16" s="6" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="17"/>
       <c r="B17" s="6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17"/>
       <c r="B18" s="6" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="17"/>
       <c r="B19" s="6" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17"/>
       <c r="B20" s="6" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="14" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="3"/>
       <c r="B23" s="3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17"/>
       <c r="B24" s="6" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="17"/>
       <c r="B25" s="6" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C25" s="7" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17"/>
       <c r="B26" s="6" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="C26" s="7" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="17"/>
       <c r="B27" s="6" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C27" s="7" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="17"/>
       <c r="B28" s="6" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C28" s="7" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="17"/>
       <c r="B29" s="6" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C29" s="7" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
     </row>
   </sheetData>
@@ -2993,7 +2942,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D28"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -3004,97 +2953,97 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="14" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>222</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="135.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
+        <v>225</v>
+      </c>
+      <c r="B6" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="C6" s="7" t="s">
         <v>227</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="s">
-        <v>229</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>230</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B7" s="7" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B8" s="7" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B9" s="7" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3102,180 +3051,166 @@
         <v>47</v>
       </c>
       <c r="B13" s="7" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>248</v>
+        <v>58</v>
       </c>
       <c r="B14" s="7" t="s">
-        <v>249</v>
+        <v>244</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>250</v>
+        <v>245</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>62</v>
+        <v>247</v>
       </c>
       <c r="B15" s="7" t="s">
-        <v>252</v>
+        <v>248</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>255</v>
+        <v>251</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>261</v>
+        <v>257</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>263</v>
+        <v>127</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>249</v>
+        <v>259</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>131</v>
+        <v>262</v>
       </c>
       <c r="B19" s="7" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
+        <v>266</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>267</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>268</v>
+      </c>
+      <c r="D20" s="7" t="s">
         <v>269</v>
       </c>
-      <c r="B20" s="7" t="s">
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="6" t="s">
         <v>270</v>
       </c>
-      <c r="C20" s="7" t="s">
+      <c r="B21" s="7" t="s">
         <v>271</v>
       </c>
-      <c r="D20" s="7" t="s">
+      <c r="C21" s="7" t="s">
         <v>272</v>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="s">
+      <c r="D21" s="7" t="s">
         <v>273</v>
       </c>
-      <c r="B21" s="7" t="s">
+    </row>
+    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="6" t="s">
         <v>274</v>
       </c>
-      <c r="C21" s="7" t="s">
+      <c r="B22" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="D21" s="7" t="s">
+      <c r="C22" s="7" t="s">
         <v>276</v>
       </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="s">
+      <c r="D22" s="7" t="s">
         <v>277</v>
       </c>
-      <c r="B22" s="7" t="s">
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="14" t="s">
         <v>278</v>
       </c>
-      <c r="C22" s="7" t="s">
+    </row>
+    <row r="25" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="18" t="s">
         <v>279</v>
       </c>
-      <c r="D22" s="7" t="s">
+      <c r="B25" s="18"/>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="2" t="s">
         <v>280</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
-        <v>281</v>
-      </c>
-      <c r="B23" s="7" t="s">
-        <v>282</v>
-      </c>
-      <c r="C23" s="7" t="s">
-        <v>283</v>
-      </c>
-      <c r="D23" s="7" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="14" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="109.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="18" t="s">
-        <v>286</v>
-      </c>
-      <c r="B26" s="18"/>
-      <c r="C26" s="18"/>
-      <c r="D26" s="18"/>
-    </row>
-    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>287</v>
-      </c>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A26:D26"/>
-    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A27:D27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>